<commit_message>
EGCH: the decree's exemption threshold is now a registered fact, so the study's own prose gate can see it
Citing decree 258 put "34.2% nitrogen" into the delivered study and the workbook, and
prose_check reported both as unreconciled — correctly, because a figure in delivered text
has to exist as a number this study holds. Registering it was not enough: the pool counts
only inputs a BUILDER CONSUMES, which is the right design, so the number had to come out
of the register rather than sit typed beside it. Both places now format it from
an_exempt_n_pct. 471 prose figures, 0 unmatched.

The fact itself is consumed by no calculation and says so in its own source string: the
duty is charged on the urea export leg and urea is not exempt.

recalc 641 of 641 formula cells, footing 51 tables clean.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017RcjXG4ETjADcoFJf123yY
</commit_message>
<xml_diff>
--- a/engine/egch_study/EGCH_Valuation_Model_05092026.xlsx
+++ b/engine/egch_study/EGCH_Valuation_Model_05092026.xlsx
@@ -2657,7 +2657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2897,16 +2897,16 @@
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Country risk priced off the sovereign's traded default swap</t>
+          <t>The new complex's granulated ammonium nitrate priced at a typed US$280/t, the weakest-sourced input in a 304-input register</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Priced off the sovereign's credit rating instead, which is the wider of the two spreads and gives a cost of capital 113 basis points higher</t>
+          <t>Priced at the SAME PRODUCT'S OWN DISCLOSED REALISED PRICE — EGP 20,000/t from note 20, which is US$408.16/t at this model's FY2024/25 rate of 49.00 (4.5269)</t>
         </is>
       </c>
       <c r="C18" s="12" t="n">
-        <v>2.509861939402812</v>
+        <v>4.526864429847856</v>
       </c>
       <c r="D18" s="11">
         <f>C18-$D$15</f>
@@ -2916,16 +2916,16 @@
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>A cost of capital that glides from its spot build to a terminal rate made from its own long-run components</t>
+          <t>Country risk priced off the sovereign's traded default swap</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>One flat spot rate applied to every explicit year and to the perpetuity</t>
+          <t>Priced off the sovereign's credit rating instead, which is the wider of the two spreads and gives a cost of capital 113 basis points higher</t>
         </is>
       </c>
       <c r="C19" s="12" t="n">
-        <v>1.437646331702388</v>
+        <v>2.509861939402812</v>
       </c>
       <c r="D19" s="11">
         <f>C19-$D$15</f>
@@ -2935,16 +2935,16 @@
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Terminal growth at the central bank's medium-term inflation target</t>
+          <t>A cost of capital that glides from its spot build to a terminal rate made from its own long-run components</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Two percentage points below it, which is negative real maintenance growth</t>
+          <t>One flat spot rate applied to every explicit year and to the perpetuity</t>
         </is>
       </c>
       <c r="C20" s="12" t="n">
-        <v>2.448134918245878</v>
+        <v>1.437646331702388</v>
       </c>
       <c r="D20" s="11">
         <f>C20-$D$15</f>
@@ -2954,16 +2954,16 @@
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>The cost of debt at the company's own disclosed rates — 19.4% on the local facility, 11.7% in dollars on the project loan carried at local-equivalent cost on the derived currency path, 24.4% in year one gliding to 13.9% at the terminal</t>
+          <t>Terminal growth at the central bank's medium-term inflation target</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Every leg floored at the 23.00% sovereign ten-year yield — the company's own facilities print no spread above the policy rate, so no spread is added</t>
+          <t>Two percentage points below it, which is negative real maintenance growth</t>
         </is>
       </c>
       <c r="C21" s="12" t="n">
-        <v>2.89382889923321</v>
+        <v>2.448134918245878</v>
       </c>
       <c r="D21" s="11">
         <f>C21-$D$15</f>
@@ -2973,16 +2973,16 @@
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Beta from the five-year weekly regression of the share against the published EGX30 index</t>
+          <t>The cost of debt at the company's own disclosed rates — 19.4% on the local facility, 11.7% in dollars on the project loan carried at local-equivalent cost on the derived currency path, 24.4% in year one gliding to 13.9% at the terminal</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>The lower bound of that regression's own 90% confidence interval</t>
+          <t>Every leg floored at the 23.00% sovereign ten-year yield — the company's own facilities print no spread above the policy rate, so no spread is added</t>
         </is>
       </c>
       <c r="C22" s="12" t="n">
-        <v>5.783551427853116</v>
+        <v>2.89382889923321</v>
       </c>
       <c r="D22" s="11">
         <f>C22-$D$15</f>
@@ -2992,16 +2992,16 @@
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Gas at the realised price the company's own loss disclosure implies</t>
+          <t>Beta from the five-year weekly regression of the share against the published EGX30 index</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>The contract formula price in the operating agreement, which is higher</t>
+          <t>The lower bound of that regression's own 90% confidence interval</t>
         </is>
       </c>
       <c r="C23" s="12" t="n">
-        <v>1.32686188934534</v>
+        <v>5.783551427853116</v>
       </c>
       <c r="D23" s="11">
         <f>C23-$D$15</f>
@@ -3011,16 +3011,16 @@
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>The new complex earning at half its derived nameplate in the terminal year</t>
+          <t>Gas at the realised price the company's own loss disclosure implies</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Seventy per cent, which is what a well-run nitrate line achieves</t>
+          <t>The contract formula price in the operating agreement, which is higher</t>
         </is>
       </c>
       <c r="C24" s="12" t="n">
-        <v>4.465410827653877</v>
+        <v>1.32686188934534</v>
       </c>
       <c r="D24" s="11">
         <f>C24-$D$15</f>
@@ -3030,16 +3030,16 @@
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>Maintenance capital expenditure at the company's own observed pre-project rate of 1.12% of revenue</t>
+          <t>The new complex earning at half its derived nameplate in the terminal year</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Replacement-rate maintenance: gross fixed assets at the disclosed 3.95% machinery depreciation rate, or 6.11% of revenue</t>
+          <t>Seventy per cent, which is what a well-run nitrate line achieves</t>
         </is>
       </c>
       <c r="C25" s="12" t="n">
-        <v>3.131128827595877</v>
+        <v>4.465410827653877</v>
       </c>
       <c r="D25" s="11">
         <f>C25-$D$15</f>
@@ -3049,16 +3049,16 @@
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>Capital maintenance charged at what replacing the plant costs today, on the 4.45-year average age the accounts MEASURE — accumulated depreciation over the year's own charge</t>
+          <t>Maintenance capital expenditure at the company's own observed pre-project rate of 1.12% of revenue</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Half the 22.1-year life the same accounts imply, 11.04 years, which is what has to be assumed where a company does not disclose enough to measure it</t>
+          <t>Replacement-rate maintenance: gross fixed assets at the disclosed 3.95% machinery depreciation rate, or 6.11% of revenue</t>
         </is>
       </c>
       <c r="C26" s="12" t="n">
-        <v>1.819746729021884</v>
+        <v>3.131128827595877</v>
       </c>
       <c r="D26" s="11">
         <f>C26-$D$15</f>
@@ -3068,16 +3068,16 @@
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Gas consumption at 1,292 cubic metres a tonne of ammonia — the rate implied by allocating three quarters of the single disclosed materials line to gas, which carries the plant's disclosed losses as well as its standard usage</t>
+          <t>Capital maintenance charged at what replacing the plant costs today, on the 4.45-year average age the accounts MEASURE — accumulated depreciation over the year's own charge</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>The auditor's own disclosed STANDARD rate of 1,200 cubic metres a tonne, which is what the plant consumes when it runs to specification and excludes the losses</t>
+          <t>Half the 22.1-year life the same accounts imply, 11.04 years, which is what has to be assumed where a company does not disclose enough to measure it</t>
         </is>
       </c>
       <c r="C27" s="12" t="n">
-        <v>4.88445528574309</v>
+        <v>1.819746729021884</v>
       </c>
       <c r="D27" s="11">
         <f>C27-$D$15</f>
@@ -3087,25 +3087,44 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Project spending anchored on the observed run rate: the nine-month actual extended to a full year</t>
+          <t>Gas consumption at 1,292 cubic metres a tonne of ammonia — the rate implied by allocating three quarters of the single disclosed materials line to gas, which carries the plant's disclosed losses as well as its standard usage</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>The faster profile the first issue of this study used, opening at EGP 3,000m</t>
+          <t>The auditor's own disclosed STANDARD rate of 1,200 cubic metres a tonne, which is what the plant consumes when it runs to specification and excludes the losses</t>
         </is>
       </c>
       <c r="C28" s="12" t="n">
-        <v>3.832876428749209</v>
+        <v>4.88445528574309</v>
       </c>
       <c r="D28" s="11">
         <f>C28-$D$15</f>
         <v/>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30" ht="39" customHeight="1">
-      <c r="A30" s="17" t="inlineStr">
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Project spending anchored on the observed run rate: the nine-month actual extended to a full year</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>The faster profile the first issue of this study used, opening at EGP 3,000m</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>3.832876428749209</v>
+      </c>
+      <c r="D29" s="11">
+        <f>C29-$D$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31" ht="39" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Each row is a complete re-run of the model through the same case machinery with one component moved and everything else held. Column C is pasted class 3 and DOES NOT REDRAW; column D is a formula against the published answer so the gap can never drift from the values beside it.</t>
         </is>
@@ -5228,7 +5247,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="48" customHeight="1">
+    <row r="50" ht="84" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
         <is>
           <t>Export duty</t>
@@ -5244,7 +5263,7 @@
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>2026 replacement of the shortfall levy with an ad-valorem duty tied to the global price. NO DECREE, MINISTRY OR RATE DOCUMENT HAS BEEN LOCATED: this rests on press reporting (Mada Masr, Edge Consultancy) as this study's own sweep register states, not on an official instrument, and it is tiered L4 for that reason while the three policy inputs above cite their decisions by number</t>
+          <t>Decree No. 258 of 2026 of the Minister of Investment and Foreign Trade, published in the Official Gazette on 25 June 2026 — 10% ad valorem on the FOB invoice value of nitrogen fertiliser exports, the invoice certified by the Chamber of Chemical Industries. It replaced a temporary US$90/t duty imposed in May 2026 for three months; the 10% carries no stated expiry. Pure ammonium nitrate above 34.2% nitrogen and free zone shipments are exempt — urea is neither. Read from two independent reports of the instrument rather than the Gazette text, which is the remaining gap in this citation</t>
         </is>
       </c>
     </row>

</xml_diff>